<commit_message>
Update Excel data and regenerate SpawnDatabase
</commit_message>
<xml_diff>
--- a/Assets/GameData/Excel/GameData.xlsx
+++ b/Assets/GameData/Excel/GameData.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t xml:space="preserve">생성수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">처치경험치</t>
   </si>
   <si>
     <t xml:space="preserve">가중치</t>
@@ -364,14 +367,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.15" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="5.25" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="4.05" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="12.45" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.05" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.05" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.45" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -399,13 +404,16 @@
       <c r="H1" s="3" t="s">
         <v>27</v>
       </c>
+      <c r="I1" s="3" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0">
         <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2" s="0">
         <v>1</v>
@@ -417,21 +425,24 @@
         <v>10</v>
       </c>
       <c r="F2" s="0">
+        <v>10</v>
+      </c>
+      <c r="G2" s="0">
         <v>60</v>
-      </c>
-      <c r="G2" s="0">
-        <v>0</v>
       </c>
       <c r="H2" s="0">
         <v>0</v>
       </c>
+      <c r="I2" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0">
         <v>1</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C3" s="0">
         <v>1</v>
@@ -443,12 +454,15 @@
         <v>8</v>
       </c>
       <c r="F3" s="0">
+        <v>20</v>
+      </c>
+      <c r="G3" s="0">
         <v>30</v>
       </c>
-      <c r="G3" s="0">
+      <c r="H3" s="0">
         <v>2.40000009536743</v>
       </c>
-      <c r="H3" s="0">
+      <c r="I3" s="0">
         <v>3.40000009536743</v>
       </c>
     </row>
@@ -457,7 +471,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" s="0">
         <v>2</v>
@@ -469,12 +483,15 @@
         <v>6</v>
       </c>
       <c r="F4" s="0">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="G4" s="0">
+        <v>10</v>
+      </c>
+      <c r="H4" s="0">
         <v>3</v>
       </c>
-      <c r="H4" s="0">
+      <c r="I4" s="0">
         <v>4.19999980926514</v>
       </c>
     </row>
@@ -483,7 +500,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" s="0">
         <v>2</v>
@@ -495,12 +512,15 @@
         <v>12</v>
       </c>
       <c r="F5" s="0">
+        <v>40</v>
+      </c>
+      <c r="G5" s="0">
         <v>50</v>
       </c>
-      <c r="G5" s="0">
+      <c r="H5" s="0">
         <v>2.59999990463257</v>
       </c>
-      <c r="H5" s="0">
+      <c r="I5" s="0">
         <v>3.79999995231628</v>
       </c>
     </row>
@@ -509,7 +529,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="0">
         <v>3</v>
@@ -524,9 +544,12 @@
         <v>50</v>
       </c>
       <c r="G6" s="0">
+        <v>50</v>
+      </c>
+      <c r="H6" s="0">
         <v>3.20000004768372</v>
       </c>
-      <c r="H6" s="0">
+      <c r="I6" s="0">
         <v>4.40000009536743</v>
       </c>
     </row>
@@ -551,16 +574,16 @@
         <v>2</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Wire data-driven dino prototype
</commit_message>
<xml_diff>
--- a/Assets/GameData/Excel/GameData.xlsx
+++ b/Assets/GameData/Excel/GameData.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="55">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -123,6 +123,63 @@
   </si>
   <si>
     <t xml:space="preserve">카메라높이</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parasaurolophus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">파라사우롤로푸스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배회형</t>
+  </si>
+  <si>
+    <t xml:space="preserve">초식</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parasaurolophus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">velociraptor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">벨로시랩터</t>
+  </si>
+  <si>
+    <t xml:space="preserve">추격형</t>
+  </si>
+  <si>
+    <t xml:space="preserve">육식</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Velociraptor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stegosaurus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">스테고사우루스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stegosaurus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">triceratops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">트리케라톱스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Triceratops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">티라노</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trex</t>
   </si>
 </sst>
 </file>
@@ -191,17 +248,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="6.3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4.05" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.6" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="5.25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -260,6 +317,151 @@
       </c>
       <c r="I2" s="0" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="0">
+        <v>1</v>
+      </c>
+      <c r="D3" s="0">
+        <v>10</v>
+      </c>
+      <c r="E3" s="0">
+        <v>2.6</v>
+      </c>
+      <c r="F3" s="0">
+        <v>1</v>
+      </c>
+      <c r="G3" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="0" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="0">
+        <v>2</v>
+      </c>
+      <c r="D4" s="0">
+        <v>20</v>
+      </c>
+      <c r="E4" s="0">
+        <v>4.2</v>
+      </c>
+      <c r="F4" s="0">
+        <v>0.9</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" s="0" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="0">
+        <v>4</v>
+      </c>
+      <c r="D5" s="0">
+        <v>40</v>
+      </c>
+      <c r="E5" s="0">
+        <v>2.2</v>
+      </c>
+      <c r="F5" s="0">
+        <v>1.4</v>
+      </c>
+      <c r="G5" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="0" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="0">
+        <v>6</v>
+      </c>
+      <c r="D6" s="0">
+        <v>60</v>
+      </c>
+      <c r="E6" s="0">
+        <v>2.4</v>
+      </c>
+      <c r="F6" s="0">
+        <v>1.6</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="0" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="0">
+        <v>10</v>
+      </c>
+      <c r="D7" s="0">
+        <v>100</v>
+      </c>
+      <c r="E7" s="0">
+        <v>3.4</v>
+      </c>
+      <c r="F7" s="0">
+        <v>2.2</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="I7" s="0" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -371,12 +573,12 @@
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.75" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="5.25" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4.05" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="4.05" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.45" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="7.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -413,28 +615,28 @@
         <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C2" s="0">
         <v>1</v>
       </c>
       <c r="D2" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="0">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F2" s="0">
         <v>10</v>
       </c>
       <c r="G2" s="0">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="H2" s="0">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I2" s="0">
-        <v>0</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="3">
@@ -442,16 +644,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="C3" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" s="0">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F3" s="0">
         <v>20</v>
@@ -460,10 +662,10 @@
         <v>30</v>
       </c>
       <c r="H3" s="0">
-        <v>2.40000009536743</v>
+        <v>3.4</v>
       </c>
       <c r="I3" s="0">
-        <v>3.40000009536743</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="4">
@@ -471,28 +673,28 @@
         <v>1</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C4" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" s="0">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F4" s="0">
         <v>30</v>
       </c>
       <c r="G4" s="0">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H4" s="0">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="I4" s="0">
-        <v>4.19999980926514</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="5">
@@ -500,28 +702,28 @@
         <v>2</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="C5" s="0">
+        <v>5</v>
+      </c>
+      <c r="D5" s="0">
+        <v>8</v>
+      </c>
+      <c r="E5" s="0">
+        <v>6</v>
+      </c>
+      <c r="F5" s="0">
+        <v>50</v>
+      </c>
+      <c r="G5" s="0">
+        <v>35</v>
+      </c>
+      <c r="H5" s="0">
         <v>2</v>
       </c>
-      <c r="D5" s="0">
-        <v>4</v>
-      </c>
-      <c r="E5" s="0">
-        <v>12</v>
-      </c>
-      <c r="F5" s="0">
-        <v>40</v>
-      </c>
-      <c r="G5" s="0">
-        <v>50</v>
-      </c>
-      <c r="H5" s="0">
-        <v>2.59999990463257</v>
-      </c>
       <c r="I5" s="0">
-        <v>3.79999995231628</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="6">
@@ -529,28 +731,28 @@
         <v>2</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="C6" s="0">
+        <v>8</v>
+      </c>
+      <c r="D6" s="0">
+        <v>12</v>
+      </c>
+      <c r="E6" s="0">
         <v>3</v>
       </c>
-      <c r="D6" s="0">
-        <v>5</v>
-      </c>
-      <c r="E6" s="0">
-        <v>10</v>
-      </c>
       <c r="F6" s="0">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G6" s="0">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="H6" s="0">
-        <v>3.20000004768372</v>
+        <v>3</v>
       </c>
       <c r="I6" s="0">
-        <v>4.40000009536743</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Optimize map10 decoration and polish growth UI
</commit_message>
<xml_diff>
--- a/Assets/GameData/Excel/GameData.xlsx
+++ b/Assets/GameData/Excel/GameData.xlsx
@@ -1159,7 +1159,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -1176,7 +1176,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C3" t="n">
         <v>1.08000004291534</v>
@@ -1193,7 +1193,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="C4" t="n">
         <v>1.1599999666214</v>
@@ -1210,7 +1210,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C5" t="n">
         <v>1.24000000953674</v>
@@ -1227,7 +1227,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="C6" t="n">
         <v>1.3199999332428</v>
@@ -1261,7 +1261,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="C8" t="n">
         <v>1.48000001907349</v>
@@ -1278,7 +1278,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="C9" t="n">
         <v>1.55999994277954</v>
@@ -1295,7 +1295,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="C10" t="n">
         <v>1.63999998569489</v>
@@ -1312,7 +1312,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="C11" t="n">
         <v>1.72000002861023</v>
@@ -1329,7 +1329,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="C12" t="n">
         <v>1.79999995231628</v>
@@ -1346,7 +1346,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="C13" t="n">
         <v>1.87999999523163</v>
@@ -1363,7 +1363,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>100</v>
+        <v>170</v>
       </c>
       <c r="C14" t="n">
         <v>1.96000003814697</v>
@@ -1380,7 +1380,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="C15" t="n">
         <v>2.03999996185303</v>
@@ -1397,7 +1397,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>100</v>
+        <v>190</v>
       </c>
       <c r="C16" t="n">
         <v>2.11999988555908</v>
@@ -1414,7 +1414,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C17" t="n">
         <v>2.20000004768372</v>
@@ -1431,7 +1431,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>100</v>
+        <v>210</v>
       </c>
       <c r="C18" t="n">
         <v>2.27999997138977</v>
@@ -1448,7 +1448,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>100</v>
+        <v>220</v>
       </c>
       <c r="C19" t="n">
         <v>2.35999989509583</v>
@@ -1465,7 +1465,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>100</v>
+        <v>230</v>
       </c>
       <c r="C20" t="n">
         <v>2.44000005722046</v>
@@ -1482,7 +1482,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>100</v>
+        <v>240</v>
       </c>
       <c r="C21" t="n">
         <v>2.51999998092651</v>

</xml_diff>